<commit_message>
Example and template workbooks carry the CircleAnswers tab; script to regenerate them
Co-authored-by: hady-dotcom <hady-dotcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/hearts-prototype/artifacts/hearts-master-sheet-template.xlsx
+++ b/hearts-prototype/artifacts/hearts-master-sheet-template.xlsx
@@ -7,15 +7,16 @@
     <sheet sheetId="1" name="Talks" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Questions" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Resources" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="CircleAnswers" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
-  <si>
-    <t>HEARTS talks. One row is one talk. talk_key is how a later import finds the same talk, so keep it stable. Leave a cell blank to leave that field as it is. Times can be seconds (90), minutes and seconds (1:30) or hours (1:02:03). status is draft, checked or live. rejected keeps a talk hidden from learners. delete removes the talk. youtube_id is the 11-character YouTube id.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="61">
+  <si>
+    <t>HEARTS talks. One row is one talk. talk_key is how a later import finds the same talk, so keep it stable. Leave a cell blank to leave that field as it is. Times can be seconds (90), minutes and seconds (1:30) or hours (1:02:03). status is draft, checked or live. rejected keeps a talk hidden from learners. delete removes the talk. youtube_id is the 11-character YouTube id. provider is youtube, vimeo or file. A Vimeo talk puts the number in vimeo_id. An uploaded film puts the media id in media_id. duration is the length in seconds. transcript is the speaker's words and is only for captions that fit in the cell (under 30,000 characters); a longer transcript is a Resources row with kind transcript and a media_id. hook_text, turn_text, land_text and transcript are the speaker's words: the kill list is not applied to them. notes is our own writing and may contain plain text such as conf=high. A hors d'oeuvre is usually 15 to 20 seconds. Up to the cap on the master desk (45 seconds unless that cap is changed) is allowed and only warned about. Shorter than 15, or longer than the cap, is refused. app_in and app_out are one continuous appetiser. hook_in and hook_out, turn_in and turn_out, land_in and land_out are up to three separate cuts. The player plays them in that order, and their lengths together stay within about 3 minutes (195 seconds).</t>
   </si>
   <si>
     <t>talk_key</t>
@@ -63,6 +64,24 @@
     <t>app_out</t>
   </si>
   <si>
+    <t>hook_in</t>
+  </si>
+  <si>
+    <t>hook_out</t>
+  </si>
+  <si>
+    <t>turn_in</t>
+  </si>
+  <si>
+    <t>turn_out</t>
+  </si>
+  <si>
+    <t>land_in</t>
+  </si>
+  <si>
+    <t>land_out</t>
+  </si>
+  <si>
     <t>hook_text</t>
   </si>
   <si>
@@ -78,7 +97,22 @@
     <t>notes</t>
   </si>
   <si>
-    <t>HEARTS pop-up questions. Name the talk with talk_key or youtube_id. Leave question_id blank to add a question, or fill it in to change that question. type is free text, multiple choice, reflection or task. status is draft or approved (approved is what learners meet in the main). source is ai or human. A blank cell leaves that field as it is. delete removes the question. Times use the same forms as the Talks tab and must fall inside the talk.</t>
+    <t>provider</t>
+  </si>
+  <si>
+    <t>vimeo_id</t>
+  </si>
+  <si>
+    <t>media_id</t>
+  </si>
+  <si>
+    <t>duration</t>
+  </si>
+  <si>
+    <t>transcript</t>
+  </si>
+  <si>
+    <t>HEARTS questions. Name the talk with talk_key or youtube_id. The export writes question_id, and an import with that id updates the same question. A row with no question_id is matched to a question on the same talk with the same time and the same text, so importing the same file again does not add a copy. Leave question_id blank only when the question is new. type is free text, multiple choice, reflection or task. status is draft or approved (approved is what learners meet). source is ai or human. A blank cell leaves that field as it is. delete removes the question. Times use the same forms as the Talks tab and must fall inside the talk. type task is an activation task: due_days is how many days the learner has (1 to 366), evidence is none, note or photo, and show_imam is yes when the imam should see it. place is popup or workbook. A workbook row is a reflection kept in the workbook rather than a pop-up in the film. Questions, choices and notes are our own writing. Notes may contain plain text such as conf=high.</t>
   </si>
   <si>
     <t>question_id</t>
@@ -117,7 +151,19 @@
     <t>source</t>
   </si>
   <si>
-    <t>HEARTS resources, one link per row. talk_key names the talk. The same talk_key and label updates that link next time. url must start with https://. kind is link or file. Leave status blank to keep the link, or put delete to remove it.</t>
+    <t>due_days</t>
+  </si>
+  <si>
+    <t>evidence</t>
+  </si>
+  <si>
+    <t>show_imam</t>
+  </si>
+  <si>
+    <t>place</t>
+  </si>
+  <si>
+    <t>HEARTS resources, one row per item. talk_key names the talk. The same talk_key and label updates that row next time. kind is link, file, summary, quote, reading, guide or transcript. url must start with https:// for a link, and for a file that is not an upload. A file row may instead put an uploaded file's number in media_id. kind transcript points at an uploaded text file (media_id) so a transcript longer than 30,000 characters can come in as a file rather than a cell; that file is copied onto the talk. summary, reading and guide are our own writing. quote and transcript are the speaker's words, so the kill list is not applied to them. A reading row is a suggestion to verify, not a link that has been checked. Leave status blank to keep the row, or put delete to remove it.</t>
   </si>
   <si>
     <t>label</t>
@@ -127,6 +173,30 @@
   </si>
   <si>
     <t>kind</t>
+  </si>
+  <si>
+    <t>body</t>
+  </si>
+  <si>
+    <t>HEARTS circle answers. One row is one answer shown under a question in “What others said” until real answers arrive. question_id is the number from the Questions tab. Leave circle_id blank to add an answer, or fill it in to change that answer. tone is warm, honest, practical, searching or quiet. length is short, medium or long. origin is ai or staff. enabled is yes or no. Put delete in status to remove the answer. Circle answers are never counted as answers.</t>
+  </si>
+  <si>
+    <t>circle_id</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>tone</t>
+  </si>
+  <si>
+    <t>length</t>
+  </si>
+  <si>
+    <t>origin</t>
+  </si>
+  <si>
+    <t>enabled</t>
   </si>
 </sst>
 </file>
@@ -517,17 +587,167 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="20" width="14" customWidth="1"/>
+    <col min="11" max="31" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+    </row>
+    <row r="2" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AE2" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:AE2"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AE1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="12" width="14" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="20" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -557,58 +777,58 @@
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -621,19 +841,69 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="16" customWidth="1"/>
-    <col min="14" max="16" width="14" customWidth="1"/>
+    <col min="1" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="48" customHeight="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="48" customHeight="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>49</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:G2"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="11" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -645,13 +915,8 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
     </row>
-    <row r="2" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -659,96 +924,37 @@
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:P2"/>
+  <autoFilter ref="A2:K2"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="5" width="14" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="48" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A2:E2"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Master sheet: optional pack column and preview choice put imported courses in a pack; opt-in push to existing pack holders, logged and undoable
Co-authored-by: hady-dotcom <hady-dotcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/hearts-prototype/artifacts/hearts-master-sheet-template.xlsx
+++ b/hearts-prototype/artifacts/hearts-master-sheet-template.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="61">
-  <si>
-    <t>HEARTS talks. One row is one talk. talk_key is how a later import finds the same talk, so keep it stable. Leave a cell blank to leave that field as it is. Times can be seconds (90), minutes and seconds (1:30) or hours (1:02:03). status is draft, checked or live. rejected keeps a talk hidden from learners. delete removes the talk. youtube_id is the 11-character YouTube id. provider is youtube, vimeo or file. A Vimeo talk puts the number in vimeo_id. An uploaded film puts the media id in media_id. duration is the length in seconds. transcript is the speaker's words and is only for captions that fit in the cell (under 30,000 characters); a longer transcript is a Resources row with kind transcript and a media_id. hook_text, turn_text, land_text and transcript are the speaker's words: the kill list is not applied to them. notes is our own writing and may contain plain text such as conf=high. A hors d'oeuvre is usually 15 to 20 seconds. Up to the cap on the master desk (45 seconds unless that cap is changed) is allowed and only warned about. Shorter than 15, or longer than the cap, is refused. app_in and app_out are one continuous appetiser. hook_in and hook_out, turn_in and turn_out, land_in and land_out are up to three separate cuts. The player plays them in that order, and their lengths together stay within about 3 minutes (195 seconds).</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="62">
+  <si>
+    <t>HEARTS talks. One row is one talk. talk_key is how a later import finds the same talk, so keep it stable. Leave a cell blank to leave that field as it is. Times can be seconds (90), minutes and seconds (1:30) or hours (1:02:03). status is draft, checked or live. rejected keeps a talk hidden from learners. delete removes the talk. youtube_id is the 11-character YouTube id. provider is youtube, vimeo or file. A Vimeo talk puts the number in vimeo_id. An uploaded film puts the media id in media_id. duration is the length in seconds. transcript is the speaker's words and is only for captions that fit in the cell (under 30,000 characters); a longer transcript is a Resources row with kind transcript and a media_id. hook_text, turn_text, land_text and transcript are the speaker's words: the kill list is not applied to them. notes is our own writing and may contain plain text such as conf=high. A hors d'oeuvre is usually 15 to 20 seconds. Up to the cap on the master desk (45 seconds unless that cap is changed) is allowed and only warned about. Shorter than 15, or longer than the cap, is refused. app_in and app_out are one continuous appetiser. hook_in and hook_out, turn_in and turn_out, land_in and land_out are up to three separate cuts. The player plays them in that order, and their lengths together stay within about 3 minutes (195 seconds). pack is optional: the name or number of a course pack that already exists, and the talk's course joins it, so people who join with that pack's codes get the course. A portal admin can only name their own portal's packs. A blank pack leaves packs as they are, and the export leaves it blank.</t>
   </si>
   <si>
     <t>talk_key</t>
@@ -110,6 +110,9 @@
   </si>
   <si>
     <t>transcript</t>
+  </si>
+  <si>
+    <t>pack</t>
   </si>
   <si>
     <t>HEARTS questions. Name the talk with talk_key or youtube_id. The export writes question_id, and an import with that id updates the same question. A row with no question_id is matched to a question on the same talk with the same time and the same text, so importing the same file again does not add a copy. Leave question_id blank only when the question is new. type is free text, multiple choice, reflection or task. status is draft or approved (approved is what learners meet). source is ai or human. A blank cell leaves that field as it is. delete removes the question. Times use the same forms as the Talks tab and must fall inside the talk. type task is an activation task: due_days is how many days the learner has (1 to 366), evidence is none, note or photo, and show_imam is yes when the imam should see it. place is popup or workbook. A workbook row is a reflection kept in the workbook rather than a pop-up in the film. Questions, choices and notes are our own writing. Notes may contain plain text such as conf=high.</t>
@@ -587,15 +590,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="31" width="14" customWidth="1"/>
+    <col min="11" max="32" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="48" customHeight="1" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="48" customHeight="1" spans="1:32" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -629,8 +632,9 @@
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
     </row>
-    <row r="2" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -724,11 +728,14 @@
       <c r="AE2" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="AF2" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AE2"/>
+  <autoFilter ref="A2:AF2"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:AE1"/>
+    <mergeCell ref="A1:AF1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -747,7 +754,7 @@
   <sheetData>
     <row r="1" ht="48" customHeight="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -777,40 +784,40 @@
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>25</v>
@@ -819,16 +826,16 @@
         <v>26</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -851,7 +858,7 @@
   <sheetData>
     <row r="1" ht="48" customHeight="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -865,19 +872,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>29</v>
@@ -903,7 +910,7 @@
   <sheetData>
     <row r="1" ht="48" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -924,28 +931,28 @@
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>25</v>

</xml_diff>